<commit_message>
working on clint registry
</commit_message>
<xml_diff>
--- a/CRM/test_data/testdata.xlsx
+++ b/CRM/test_data/testdata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/eb01e6d76ae9d0d2/SaanviTechCRM/CRM/test_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{BB610137-23FA-4518-837F-A73E4AC39091}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D252ED79-A341-4E59-821A-CD19BA8DF3B1}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{BB610137-23FA-4518-837F-A73E4AC39091}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{84F38F3C-B014-4253-B391-B1284E8C034C}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
   <si>
     <t>business_email</t>
   </si>
@@ -68,12 +68,6 @@
     <t>BRJPV8284J</t>
   </si>
   <si>
-    <t>run</t>
-  </si>
-  <si>
-    <t>Y</t>
-  </si>
-  <si>
     <t>vinuthaacharya26@gmail.com</t>
   </si>
   <si>
@@ -87,6 +81,24 @@
   </si>
   <si>
     <t>whatsapp_group</t>
+  </si>
+  <si>
+    <t>YES</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>test</t>
+  </si>
+  <si>
+    <t>ABJPV8284J</t>
+  </si>
+  <si>
+    <t>vinutha.a@saanvitechin.com</t>
+  </si>
+  <si>
+    <t>Status</t>
   </si>
 </sst>
 </file>
@@ -486,7 +498,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24C8E921-6ACA-4AB0-8C34-6351D8E2CB95}">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="26.28515625" customWidth="1"/>
@@ -499,7 +511,7 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="B1" t="s">
         <v>8</v>
@@ -508,24 +520,24 @@
         <v>9</v>
       </c>
       <c r="D1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E1" t="s">
         <v>10</v>
       </c>
       <c r="F1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="G1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" t="s">
         <v>14</v>
-      </c>
-      <c r="B2" t="s">
-        <v>16</v>
       </c>
       <c r="C2" t="s">
         <v>11</v>
@@ -534,15 +546,36 @@
         <v>12</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F2">
         <v>9876876732</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3">
+        <v>9876832567</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="E2" r:id="rId1" xr:uid="{6553A644-DDA2-46C0-B879-B808C051BBBF}"/>
+    <hyperlink ref="E3" r:id="rId2" xr:uid="{2ABDEF37-06C6-4A2B-BADD-917ABF8E0074}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>